<commit_message>
Remove aba TabelaSIGITEC e valida analises
</commit_message>
<xml_diff>
--- a/data/EV_00000.xlsx
+++ b/data/EV_00000.xlsx
@@ -10,10 +10,9 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0284FA76-329B-4ED3-B877-FF9446854B3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{A7CC8E1A-EC12-4A9C-BA80-6AACD1CD2892}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{A7CC8E1A-EC12-4A9C-BA80-6AACD1CD2892}"/>
   </bookViews>
   <sheets>
-    <sheet name="TabelaSIGITEC" sheetId="6" r:id="rId1"/>
     <sheet name="Projeto" sheetId="3" r:id="rId2"/>
     <sheet name="Equipe" sheetId="2" r:id="rId3"/>
     <sheet name="Atividades" sheetId="1" r:id="rId4"/>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="118">
   <si>
     <t>wu</t>
   </si>
@@ -114,186 +113,6 @@
     <t>Descrição Atividade 7</t>
   </si>
   <si>
-    <t>Nivel</t>
-  </si>
-  <si>
-    <t>Valor mensal</t>
-  </si>
-  <si>
-    <t>Funcao</t>
-  </si>
-  <si>
-    <t>Nível</t>
-  </si>
-  <si>
-    <t>Peso relativo</t>
-  </si>
-  <si>
-    <t>Critérios</t>
-  </si>
-  <si>
-    <t>DESCRIÇÃO</t>
-  </si>
-  <si>
-    <t>R$</t>
-  </si>
-  <si>
-    <t>Auxiliar Administrativo I</t>
-  </si>
-  <si>
-    <t>Auxiliar administrativo</t>
-  </si>
-  <si>
-    <t>Bolsa Graduação</t>
-  </si>
-  <si>
-    <t>Auxiliar Administrativo II</t>
-  </si>
-  <si>
-    <t>Auxiliar administrativo com mais de 10 (dez) anos de experiência profissional</t>
-  </si>
-  <si>
-    <t>Bolsa Mestrando</t>
-  </si>
-  <si>
-    <t>Auxiliar Técnico</t>
-  </si>
-  <si>
-    <t>Profissional com ensino fundamental completo e mais de 10 (dez) anos de experiência profissional</t>
-  </si>
-  <si>
-    <t>Bolsa Doutorando</t>
-  </si>
-  <si>
-    <t>Pesquisador</t>
-  </si>
-  <si>
-    <t>Doutor I</t>
-  </si>
-  <si>
-    <t>Doutor há no mínimo 4 (quatro) anos com experiência na execução de projetos científico-tecnológicos</t>
-  </si>
-  <si>
-    <t>Bolsa PósDoc</t>
-  </si>
-  <si>
-    <t>Doutor II</t>
-  </si>
-  <si>
-    <t>Doutor há no mínimo 10 (dez) anos com experiência na execução de projetos científico-tecnológicos</t>
-  </si>
-  <si>
-    <t>Pesquisador A</t>
-  </si>
-  <si>
-    <t>Pesquisador Visitante</t>
-  </si>
-  <si>
-    <t>Doutor III</t>
-  </si>
-  <si>
-    <t>Doutor há no mínimo 15 (quinze) anos com experiência em orientação de doutorando, há no mínimo 12 (doze) anos, em instituições estrangeiras no tema de pesquisa em referência</t>
-  </si>
-  <si>
-    <t>Pesquisador B</t>
-  </si>
-  <si>
-    <t>Mestre I</t>
-  </si>
-  <si>
-    <t>Mestre há no mínimo 2 (dois) anos com experiência na execução de projetos científico-tecnológicos</t>
-  </si>
-  <si>
-    <t>Pesquisador C</t>
-  </si>
-  <si>
-    <t>Mestre II</t>
-  </si>
-  <si>
-    <t>Mestre há no mínimo 5 (cinco) anos com experiência na execução de projetos científico-tecnológicos</t>
-  </si>
-  <si>
-    <t>Pesquisador D</t>
-  </si>
-  <si>
-    <t>Bolsista Graduando</t>
-  </si>
-  <si>
-    <t>Nível Médio / Graduação</t>
-  </si>
-  <si>
-    <t>Aluno de nível superior ou profissional de nível médio</t>
-  </si>
-  <si>
-    <t>Pesquisador E</t>
-  </si>
-  <si>
-    <t>Pesquisador I</t>
-  </si>
-  <si>
-    <t>Nível superior completo com experiência na coordenação de projetos, ou com 6 (seis) anos de experiência profissional</t>
-  </si>
-  <si>
-    <t>Pesquisador F</t>
-  </si>
-  <si>
-    <t>Pesquisador II</t>
-  </si>
-  <si>
-    <t>Nível superior completo com 5 (cinco) anos de experiência na coordenação de projetos, ou com 12 (doze) anos de experiência profissional</t>
-  </si>
-  <si>
-    <t>Pesquisador G</t>
-  </si>
-  <si>
-    <t>Profissional Júnior</t>
-  </si>
-  <si>
-    <t>Nível superior completo</t>
-  </si>
-  <si>
-    <t>Pesquisador H</t>
-  </si>
-  <si>
-    <t>Profissional Pleno</t>
-  </si>
-  <si>
-    <t>Nível superior completo com mais de 5 (cinco) anos de experiência profissional</t>
-  </si>
-  <si>
-    <t>Profissional Sênior</t>
-  </si>
-  <si>
-    <t>Nível superior completo com mais de 10 (dez) anos de experiência profissional</t>
-  </si>
-  <si>
-    <t>Pesquisador J</t>
-  </si>
-  <si>
-    <t>Recém-Doutor</t>
-  </si>
-  <si>
-    <t>Doutorado completo</t>
-  </si>
-  <si>
-    <t>Recém-Mestre</t>
-  </si>
-  <si>
-    <t>Mestrado completo</t>
-  </si>
-  <si>
-    <t>Técnico Nível Médio I</t>
-  </si>
-  <si>
-    <t>Técnico de nível médio</t>
-  </si>
-  <si>
-    <t>Técnico Nível Médio II</t>
-  </si>
-  <si>
-    <t>Técnico de nível médio com mais de 10 (dez) anos de experiência profissional</t>
-  </si>
-  <si>
     <t>expected_duration</t>
   </si>
   <si>
@@ -367,12 +186,6 @@
   </si>
   <si>
     <t>Name 04</t>
-  </si>
-  <si>
-    <t>Profile</t>
-  </si>
-  <si>
-    <t>em wu/h</t>
   </si>
   <si>
     <t>member_expected_wu</t>
@@ -1821,489 +1634,6 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4CED948-9ED8-431E-B14F-41D87629B372}">
-  <dimension ref="A1:K22"/>
-  <sheetFormatPr defaultRowHeight="18"/>
-  <cols>
-    <col min="1" max="1" width="25.25" style="42" customWidth="1"/>
-    <col min="2" max="2" width="34.375" style="22" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.375" style="49" customWidth="1"/>
-    <col min="4" max="4" width="18.75" style="49" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="71.75" style="22" customWidth="1"/>
-    <col min="6" max="6" width="4.75" style="22" customWidth="1"/>
-    <col min="7" max="7" width="32.375" style="42" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.375" style="44" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="14.375" style="35" customWidth="1"/>
-    <col min="11" max="11" width="14.375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.25" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" ht="18.75" thickBot="1">
-      <c r="A1" s="18"/>
-      <c r="B1" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="21"/>
-      <c r="G1" s="23" t="s">
-        <v>25</v>
-      </c>
-      <c r="H1" s="23"/>
-      <c r="I1"/>
-      <c r="J1"/>
-    </row>
-    <row r="2" spans="1:11">
-      <c r="A2" s="24" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" s="26" t="s">
-        <v>109</v>
-      </c>
-      <c r="D2" s="26" t="s">
-        <v>28</v>
-      </c>
-      <c r="E2" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="G2" s="28" t="s">
-        <v>30</v>
-      </c>
-      <c r="H2" s="28" t="s">
-        <v>31</v>
-      </c>
-      <c r="I2"/>
-      <c r="J2"/>
-    </row>
-    <row r="3" spans="1:11">
-      <c r="A3" s="29"/>
-      <c r="B3" s="30" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" s="26">
-        <f>D3*$C$8</f>
-        <v>30</v>
-      </c>
-      <c r="D3" s="50">
-        <v>0.1</v>
-      </c>
-      <c r="E3" s="31" t="s">
-        <v>33</v>
-      </c>
-      <c r="G3" s="32" t="s">
-        <v>34</v>
-      </c>
-      <c r="H3" s="32">
-        <v>1092</v>
-      </c>
-      <c r="I3" s="33"/>
-      <c r="J3" s="33"/>
-      <c r="K3" s="33"/>
-    </row>
-    <row r="4" spans="1:11" ht="36.75" thickBot="1">
-      <c r="A4" s="29"/>
-      <c r="B4" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" s="26">
-        <f t="shared" ref="C4:C20" si="0">D4*$C$8</f>
-        <v>30</v>
-      </c>
-      <c r="D4" s="50">
-        <v>0.1</v>
-      </c>
-      <c r="E4" s="31" t="s">
-        <v>36</v>
-      </c>
-      <c r="G4" s="32" t="s">
-        <v>37</v>
-      </c>
-      <c r="H4" s="32">
-        <v>2996</v>
-      </c>
-      <c r="I4" s="33"/>
-      <c r="J4" s="33"/>
-    </row>
-    <row r="5" spans="1:11" ht="36.75" thickBot="1">
-      <c r="A5" s="34"/>
-      <c r="B5" s="30" t="s">
-        <v>38</v>
-      </c>
-      <c r="C5" s="26">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-      <c r="D5" s="50">
-        <v>0.1</v>
-      </c>
-      <c r="E5" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="G5" s="32" t="s">
-        <v>40</v>
-      </c>
-      <c r="H5" s="32">
-        <v>4158</v>
-      </c>
-      <c r="I5" s="33"/>
-      <c r="J5" s="33"/>
-    </row>
-    <row r="6" spans="1:11" ht="36.75" thickBot="1">
-      <c r="A6" s="34" t="s">
-        <v>41</v>
-      </c>
-      <c r="B6" s="30" t="s">
-        <v>42</v>
-      </c>
-      <c r="C6" s="26">
-        <f t="shared" si="0"/>
-        <v>255</v>
-      </c>
-      <c r="D6" s="50">
-        <v>0.85</v>
-      </c>
-      <c r="E6" s="31" t="s">
-        <v>43</v>
-      </c>
-      <c r="G6" s="32" t="s">
-        <v>44</v>
-      </c>
-      <c r="H6" s="32"/>
-      <c r="J6"/>
-    </row>
-    <row r="7" spans="1:11" ht="36.75" thickBot="1">
-      <c r="A7" s="34" t="s">
-        <v>41</v>
-      </c>
-      <c r="B7" s="30" t="s">
-        <v>45</v>
-      </c>
-      <c r="C7" s="26">
-        <f t="shared" si="0"/>
-        <v>300</v>
-      </c>
-      <c r="D7" s="50">
-        <v>1</v>
-      </c>
-      <c r="E7" s="31" t="s">
-        <v>46</v>
-      </c>
-      <c r="G7" s="32" t="s">
-        <v>47</v>
-      </c>
-      <c r="H7" s="32"/>
-      <c r="J7"/>
-    </row>
-    <row r="8" spans="1:11" ht="72.75" thickBot="1">
-      <c r="A8" s="36" t="s">
-        <v>48</v>
-      </c>
-      <c r="B8" s="37" t="s">
-        <v>49</v>
-      </c>
-      <c r="C8" s="50">
-        <v>300</v>
-      </c>
-      <c r="D8" s="50">
-        <v>1</v>
-      </c>
-      <c r="E8" s="31" t="s">
-        <v>50</v>
-      </c>
-      <c r="G8" s="32" t="s">
-        <v>51</v>
-      </c>
-      <c r="H8" s="32">
-        <v>10758.88</v>
-      </c>
-      <c r="J8"/>
-    </row>
-    <row r="9" spans="1:11" ht="36.75" thickBot="1">
-      <c r="A9" s="34" t="s">
-        <v>41</v>
-      </c>
-      <c r="B9" s="30" t="s">
-        <v>52</v>
-      </c>
-      <c r="C9" s="26">
-        <f t="shared" si="0"/>
-        <v>120</v>
-      </c>
-      <c r="D9" s="50">
-        <v>0.4</v>
-      </c>
-      <c r="E9" s="31" t="s">
-        <v>53</v>
-      </c>
-      <c r="G9" s="32" t="s">
-        <v>54</v>
-      </c>
-      <c r="H9" s="32">
-        <v>9682.99</v>
-      </c>
-      <c r="J9"/>
-    </row>
-    <row r="10" spans="1:11" ht="36.75" thickBot="1">
-      <c r="A10" s="34" t="s">
-        <v>41</v>
-      </c>
-      <c r="B10" s="30" t="s">
-        <v>55</v>
-      </c>
-      <c r="C10" s="26">
-        <f t="shared" si="0"/>
-        <v>180</v>
-      </c>
-      <c r="D10" s="50">
-        <v>0.6</v>
-      </c>
-      <c r="E10" s="31" t="s">
-        <v>56</v>
-      </c>
-      <c r="G10" s="32" t="s">
-        <v>57</v>
-      </c>
-      <c r="H10" s="32">
-        <v>8607.1</v>
-      </c>
-      <c r="J10"/>
-    </row>
-    <row r="11" spans="1:11" ht="36">
-      <c r="A11" s="38" t="s">
-        <v>58</v>
-      </c>
-      <c r="B11" s="30" t="s">
-        <v>59</v>
-      </c>
-      <c r="C11" s="26">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-      <c r="D11" s="50">
-        <v>0.1</v>
-      </c>
-      <c r="E11" s="31" t="s">
-        <v>60</v>
-      </c>
-      <c r="G11" s="32" t="s">
-        <v>61</v>
-      </c>
-      <c r="H11" s="32">
-        <v>7531.22</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="54">
-      <c r="A12" s="39"/>
-      <c r="B12" s="40" t="s">
-        <v>62</v>
-      </c>
-      <c r="C12" s="26">
-        <f t="shared" si="0"/>
-        <v>210</v>
-      </c>
-      <c r="D12" s="50">
-        <v>0.7</v>
-      </c>
-      <c r="E12" s="31" t="s">
-        <v>63</v>
-      </c>
-      <c r="G12" s="32" t="s">
-        <v>64</v>
-      </c>
-      <c r="H12" s="32">
-        <v>6455.33</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="54">
-      <c r="A13" s="39"/>
-      <c r="B13" s="40" t="s">
-        <v>65</v>
-      </c>
-      <c r="C13" s="26">
-        <f t="shared" si="0"/>
-        <v>240</v>
-      </c>
-      <c r="D13" s="50">
-        <v>0.8</v>
-      </c>
-      <c r="E13" s="31" t="s">
-        <v>66</v>
-      </c>
-      <c r="G13" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="H13" s="32">
-        <v>8921.61</v>
-      </c>
-      <c r="J13"/>
-    </row>
-    <row r="14" spans="1:11">
-      <c r="A14" s="39" t="s">
-        <v>41</v>
-      </c>
-      <c r="B14" s="40" t="s">
-        <v>68</v>
-      </c>
-      <c r="C14" s="26">
-        <f t="shared" si="0"/>
-        <v>150</v>
-      </c>
-      <c r="D14" s="50">
-        <v>0.5</v>
-      </c>
-      <c r="E14" s="31" t="s">
-        <v>69</v>
-      </c>
-      <c r="G14" s="32" t="s">
-        <v>70</v>
-      </c>
-      <c r="H14" s="32">
-        <v>6691.21</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="36">
-      <c r="A15" s="39" t="s">
-        <v>41</v>
-      </c>
-      <c r="B15" s="40" t="s">
-        <v>71</v>
-      </c>
-      <c r="C15" s="26">
-        <f t="shared" si="0"/>
-        <v>210</v>
-      </c>
-      <c r="D15" s="50">
-        <v>0.7</v>
-      </c>
-      <c r="E15" s="31" t="s">
-        <v>72</v>
-      </c>
-      <c r="G15" s="32" t="s">
-        <v>62</v>
-      </c>
-      <c r="H15" s="32">
-        <v>5379.44</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="36">
-      <c r="A16" s="39" t="s">
-        <v>41</v>
-      </c>
-      <c r="B16" s="40" t="s">
-        <v>73</v>
-      </c>
-      <c r="C16" s="26">
-        <f t="shared" si="0"/>
-        <v>240</v>
-      </c>
-      <c r="D16" s="50">
-        <v>0.8</v>
-      </c>
-      <c r="E16" s="31" t="s">
-        <v>74</v>
-      </c>
-      <c r="G16" s="32" t="s">
-        <v>75</v>
-      </c>
-      <c r="H16" s="32">
-        <v>3227.66</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10">
-      <c r="A17" s="39" t="s">
-        <v>41</v>
-      </c>
-      <c r="B17" s="40" t="s">
-        <v>76</v>
-      </c>
-      <c r="C17" s="26">
-        <f t="shared" si="0"/>
-        <v>210</v>
-      </c>
-      <c r="D17" s="50">
-        <v>0.7</v>
-      </c>
-      <c r="E17" s="31" t="s">
-        <v>77</v>
-      </c>
-      <c r="G17" s="32" t="s">
-        <v>48</v>
-      </c>
-      <c r="H17" s="32"/>
-      <c r="I17" s="41"/>
-      <c r="J17" s="41"/>
-    </row>
-    <row r="18" spans="1:10">
-      <c r="A18" s="39" t="s">
-        <v>41</v>
-      </c>
-      <c r="B18" s="40" t="s">
-        <v>78</v>
-      </c>
-      <c r="C18" s="26">
-        <f t="shared" si="0"/>
-        <v>105</v>
-      </c>
-      <c r="D18" s="50">
-        <v>0.35</v>
-      </c>
-      <c r="E18" s="31" t="s">
-        <v>79</v>
-      </c>
-      <c r="H18" s="43"/>
-      <c r="I18" s="41"/>
-      <c r="J18" s="41"/>
-    </row>
-    <row r="19" spans="1:10">
-      <c r="A19" s="39" t="s">
-        <v>41</v>
-      </c>
-      <c r="B19" s="40" t="s">
-        <v>80</v>
-      </c>
-      <c r="C19" s="26">
-        <f t="shared" si="0"/>
-        <v>45</v>
-      </c>
-      <c r="D19" s="50">
-        <v>0.15</v>
-      </c>
-      <c r="E19" s="31" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="36.75" thickBot="1">
-      <c r="A20" s="45" t="s">
-        <v>41</v>
-      </c>
-      <c r="B20" s="46" t="s">
-        <v>82</v>
-      </c>
-      <c r="C20" s="47">
-        <f t="shared" si="0"/>
-        <v>75</v>
-      </c>
-      <c r="D20" s="51">
-        <v>0.25</v>
-      </c>
-      <c r="E20" s="48" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="23.25">
-      <c r="C22" s="80" t="s">
-        <v>110</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F696936E-B939-4714-9610-63788CF7A0B8}">
   <dimension ref="A1:J22"/>
@@ -2329,19 +1659,19 @@
         <v>10</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>88</v>
+        <v>28</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>93</v>
+        <v>33</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>92</v>
+        <v>32</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>4</v>
@@ -2379,40 +1709,40 @@
     </row>
     <row r="3" spans="1:9">
       <c r="C3" s="1" t="s">
-        <v>91</v>
+        <v>31</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>89</v>
+        <v>29</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>133</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="C4" s="57" t="s">
-        <v>139</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="57" t="s">
-        <v>85</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="57" t="s">
-        <v>87</v>
+        <v>27</v>
       </c>
       <c r="B7" s="1">
         <v>4.4000000000000004</v>
       </c>
       <c r="C7" s="57" t="s">
-        <v>86</v>
+        <v>26</v>
       </c>
       <c r="D7" s="57"/>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="57" t="s">
-        <v>104</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -2445,10 +1775,10 @@
         <v>16</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>127</v>
+        <v>65</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>140</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -2626,7 +1956,7 @@
         <v>22</v>
       </c>
       <c r="C17" s="53" t="s">
-        <v>178</v>
+        <v>116</v>
       </c>
       <c r="D17" s="14">
         <f>E16</f>
@@ -2696,7 +2026,7 @@
       <c r="E19" s="61"/>
       <c r="F19" s="61"/>
       <c r="G19" s="69" t="s">
-        <v>130</v>
+        <v>68</v>
       </c>
       <c r="H19" s="72">
         <f>SUM(H12:H18)</f>
@@ -2709,12 +2039,12 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="57" t="s">
-        <v>131</v>
+        <v>69</v>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="57" t="s">
-        <v>128</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -2750,37 +2080,37 @@
         <v>1</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>114</v>
+        <v>52</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>115</v>
+        <v>53</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>120</v>
+        <v>58</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>116</v>
+        <v>54</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>117</v>
+        <v>55</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>118</v>
+        <v>56</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>111</v>
+        <v>49</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>98</v>
+        <v>38</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>99</v>
+        <v>39</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>101</v>
+        <v>41</v>
       </c>
       <c r="M1" s="9" t="s">
         <v>11</v>
@@ -2793,7 +2123,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="55" t="s">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="C2" s="55">
         <v>12</v>
@@ -2840,7 +2170,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="55" t="s">
-        <v>106</v>
+        <v>46</v>
       </c>
       <c r="C3" s="55">
         <v>12</v>
@@ -2888,7 +2218,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="55" t="s">
-        <v>107</v>
+        <v>47</v>
       </c>
       <c r="C4" s="55">
         <v>6</v>
@@ -2936,7 +2266,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="55" t="s">
-        <v>108</v>
+        <v>48</v>
       </c>
       <c r="C5" s="55">
         <v>12</v>
@@ -2981,16 +2311,16 @@
     </row>
     <row r="6" spans="1:16">
       <c r="C6" s="1" t="s">
-        <v>97</v>
+        <v>37</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>86</v>
+        <v>26</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>138</v>
+        <v>76</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>129</v>
+        <v>67</v>
       </c>
       <c r="H6" s="67">
         <f>SUM(H2:H5)</f>
@@ -3019,16 +2349,16 @@
     <row r="9" spans="1:16">
       <c r="C9" s="12"/>
       <c r="D9" s="12" t="s">
-        <v>94</v>
+        <v>34</v>
       </c>
       <c r="E9" s="60" t="s">
-        <v>95</v>
+        <v>35</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>96</v>
+        <v>36</v>
       </c>
       <c r="G9" s="60" t="s">
-        <v>124</v>
+        <v>62</v>
       </c>
       <c r="H9" s="12" t="s">
         <v>0</v>
@@ -3045,32 +2375,32 @@
     </row>
     <row r="11" spans="1:16">
       <c r="A11" s="57" t="s">
-        <v>119</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12" spans="1:16">
       <c r="A12" s="57" t="s">
-        <v>121</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:16">
       <c r="A13" s="57" t="s">
-        <v>122</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:16">
       <c r="A14" s="57" t="s">
-        <v>123</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15" spans="1:16">
       <c r="A15" s="57" t="s">
-        <v>125</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:16">
       <c r="A16" s="57" t="s">
-        <v>112</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:16">
@@ -3078,7 +2408,7 @@
     </row>
     <row r="18" spans="1:16">
       <c r="A18" s="57" t="s">
-        <v>113</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" spans="1:16">
@@ -3090,7 +2420,7 @@
       <c r="D20"/>
       <c r="E20"/>
       <c r="F20" s="62" t="s">
-        <v>135</v>
+        <v>73</v>
       </c>
       <c r="G20" s="62"/>
       <c r="H20" s="62"/>
@@ -3126,7 +2456,7 @@
     </row>
     <row r="22" spans="1:16" ht="15">
       <c r="B22" s="65" t="s">
-        <v>103</v>
+        <v>43</v>
       </c>
       <c r="C22" s="65"/>
       <c r="D22" s="65"/>
@@ -3144,7 +2474,7 @@
     </row>
     <row r="23" spans="1:16" ht="15">
       <c r="B23" s="62" t="s">
-        <v>126</v>
+        <v>64</v>
       </c>
       <c r="C23" s="62"/>
       <c r="D23" s="62"/>
@@ -3187,7 +2517,7 @@
         <v>4</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>127</v>
+        <v>65</v>
       </c>
       <c r="L24"/>
       <c r="O24"/>
@@ -3481,7 +2811,7 @@
     </row>
     <row r="32" spans="1:16">
       <c r="A32" s="11" t="s">
-        <v>132</v>
+        <v>70</v>
       </c>
       <c r="B32" s="61">
         <f>SUM(B25:B31)</f>
@@ -3525,7 +2855,7 @@
     </row>
     <row r="33" spans="1:16">
       <c r="A33" s="11" t="s">
-        <v>134</v>
+        <v>72</v>
       </c>
       <c r="B33" s="1">
         <f>SUMIF($A$2:$A$5,B24,$D$2:$D$5)-B32</f>
@@ -3573,7 +2903,7 @@
       <c r="H34" s="1"/>
       <c r="I34" s="1"/>
       <c r="J34" s="16" t="s">
-        <v>102</v>
+        <v>42</v>
       </c>
       <c r="L34"/>
       <c r="O34"/>
@@ -3593,7 +2923,7 @@
     <row r="36" spans="1:16">
       <c r="A36" s="74"/>
       <c r="B36" s="75" t="s">
-        <v>136</v>
+        <v>74</v>
       </c>
       <c r="C36" s="75"/>
       <c r="D36" s="75"/>
@@ -3674,7 +3004,7 @@
         <v>240</v>
       </c>
       <c r="C39" s="100" t="s">
-        <v>137</v>
+        <v>75</v>
       </c>
       <c r="D39" s="101"/>
       <c r="E39" s="101"/>
@@ -3845,7 +3175,7 @@
         <v>5</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>156</v>
+        <v>94</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>14</v>
@@ -3854,124 +3184,124 @@
         <v>16</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="G1" s="92" t="s">
+        <v>80</v>
+      </c>
+      <c r="H1" s="93" t="s">
+        <v>81</v>
+      </c>
+      <c r="I1" s="92" t="s">
+        <v>82</v>
+      </c>
+      <c r="J1" s="92" t="s">
+        <v>79</v>
+      </c>
+      <c r="K1" s="88" t="s">
+        <v>89</v>
+      </c>
+      <c r="L1" s="88" t="s">
+        <v>90</v>
+      </c>
+      <c r="M1" s="89" t="s">
+        <v>91</v>
+      </c>
+      <c r="N1" s="88" t="s">
+        <v>92</v>
+      </c>
+      <c r="O1" s="88" t="s">
+        <v>93</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="R1" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="S1" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="T1" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="U1" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="V1" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="W1" s="96" t="s">
+        <v>101</v>
+      </c>
+      <c r="X1" s="96" t="s">
+        <v>102</v>
+      </c>
+      <c r="Y1" s="96" t="s">
+        <v>103</v>
+      </c>
+      <c r="Z1" s="96" t="s">
+        <v>104</v>
+      </c>
+      <c r="AA1" s="96" t="s">
+        <v>105</v>
+      </c>
+      <c r="AB1" s="96" t="s">
+        <v>106</v>
+      </c>
+      <c r="AC1" s="82" t="s">
+        <v>110</v>
+      </c>
+      <c r="AD1" s="82" t="s">
+        <v>111</v>
+      </c>
+      <c r="AE1" s="82" t="s">
+        <v>112</v>
+      </c>
+      <c r="AF1" s="82" t="s">
+        <v>113</v>
+      </c>
+      <c r="AG1" s="82" t="s">
+        <v>114</v>
+      </c>
+      <c r="AH1" s="83" t="s">
+        <v>115</v>
+      </c>
+      <c r="AI1" s="90" t="s">
+        <v>83</v>
+      </c>
+      <c r="AJ1" s="90" t="s">
         <v>84</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="G1" s="92" t="s">
-        <v>142</v>
-      </c>
-      <c r="H1" s="93" t="s">
-        <v>143</v>
-      </c>
-      <c r="I1" s="92" t="s">
-        <v>144</v>
-      </c>
-      <c r="J1" s="92" t="s">
-        <v>141</v>
-      </c>
-      <c r="K1" s="88" t="s">
-        <v>151</v>
-      </c>
-      <c r="L1" s="88" t="s">
-        <v>152</v>
-      </c>
-      <c r="M1" s="89" t="s">
-        <v>153</v>
-      </c>
-      <c r="N1" s="88" t="s">
-        <v>154</v>
-      </c>
-      <c r="O1" s="88" t="s">
-        <v>155</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q1" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="R1" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="S1" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="T1" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="V1" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="W1" s="96" t="s">
-        <v>163</v>
-      </c>
-      <c r="X1" s="96" t="s">
-        <v>164</v>
-      </c>
-      <c r="Y1" s="96" t="s">
-        <v>165</v>
-      </c>
-      <c r="Z1" s="96" t="s">
-        <v>166</v>
-      </c>
-      <c r="AA1" s="96" t="s">
-        <v>167</v>
-      </c>
-      <c r="AB1" s="96" t="s">
-        <v>168</v>
-      </c>
-      <c r="AC1" s="82" t="s">
-        <v>172</v>
-      </c>
-      <c r="AD1" s="82" t="s">
-        <v>173</v>
-      </c>
-      <c r="AE1" s="82" t="s">
-        <v>174</v>
-      </c>
-      <c r="AF1" s="82" t="s">
-        <v>175</v>
-      </c>
-      <c r="AG1" s="82" t="s">
-        <v>176</v>
-      </c>
-      <c r="AH1" s="83" t="s">
-        <v>177</v>
-      </c>
-      <c r="AI1" s="90" t="s">
-        <v>145</v>
-      </c>
-      <c r="AJ1" s="90" t="s">
-        <v>146</v>
-      </c>
       <c r="AK1" s="90" t="s">
-        <v>147</v>
+        <v>85</v>
       </c>
       <c r="AL1" s="90" t="s">
-        <v>148</v>
+        <v>86</v>
       </c>
       <c r="AM1" s="90" t="s">
-        <v>149</v>
+        <v>87</v>
       </c>
       <c r="AN1" s="91" t="s">
-        <v>150</v>
+        <v>88</v>
       </c>
       <c r="AO1" s="97" t="s">
-        <v>169</v>
+        <v>107</v>
       </c>
       <c r="AP1" s="97" t="s">
-        <v>170</v>
+        <v>108</v>
       </c>
       <c r="AQ1" s="97" t="s">
-        <v>171</v>
+        <v>109</v>
       </c>
       <c r="AR1" s="97" t="s">
-        <v>179</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:44">

</xml_diff>